<commit_message>
Pass2: add confirmed LWDA PAGA findings (Track 1)
Three confirmed PAGA notices (Board and Brew Restaurant Group LLC 2022;
OSB&B LLC 2022 -> SD Superior 37-2023-00005528-CU-OE-CTL; CYPRESSBNB LLC
2026). Update Employment tab, delta memo Q10, exceptions.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LNcNsZWWbrzPfifpECK5UT
</commit_message>
<xml_diff>
--- a/BoardAndBrew_PublicRecords_Pass2_20260725/_Outputs/BoardAndBrew_EntityMap_Pass2.xlsx
+++ b/BoardAndBrew_PublicRecords_Pass2_20260725/_Outputs/BoardAndBrew_EntityMap_Pass2.xlsx
@@ -3259,7 +3259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3311,32 +3311,32 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>DOL WHD (enforcedata.dol.gov)</t>
+          <t>CA LWDA PAGA</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>JJ&amp;N / BBRG / franchisee LLCs</t>
+          <t>Board and Brew Restaurant Group, LLC (franchisor)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>No matching enforcement record surfaced via search</t>
+          <t>PAGA Notice, filed 2022-07-11; San Clemente; 100 employees; plaintiff Kaley Cruz (Bibiyan Law Group); no court complaint</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LWDA-CM-894611-22</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>GAP (null; DB is JS — not confirmed exhaustively)</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>https://enforcedata.dol.gov/</t>
+          <t>https://cadir.my.salesforce-sites.com/PagaSearch</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -3353,27 +3353,27 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>all subjects</t>
+          <t>OSB&amp;B, LLC (franchisee)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>No PAGA notice surfaced via search</t>
+          <t>PAGA Notice 2022-12-05 + Court Complaint 2023-02-14; Cardiff-by-the-Sea; 150 employees; plaintiff Brandy Harman (Lawyers for Justice); SD Superior case 37-2023-00005528-CU-OE-CTL</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LWDA-CM-922795-22</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>GAP (portal JS)</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>https://cadir.lwda.ca.gov/</t>
+          <t>https://cadir.my.salesforce-sites.com/PagaSearch</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3385,32 +3385,32 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CA DLSE / Labor Commissioner</t>
+          <t>CA LWDA PAGA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>all subjects</t>
+          <t>CYPRESSBNB LLC dba Board and Brew (franchisee, not on task list)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>No wage judgment surfaced via search</t>
+          <t>PAGA Notice, filed 2026-01-02; Cypress; 15 employees; plaintiff Ana Karen Martinez Ramirez (Lipeles Law); no court complaint yet</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LWDA-CM-1147303-26</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>GAP (portal JS)</t>
+          <t>CONFIRMED</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>https://www.dir.ca.gov/dlse/</t>
+          <t>https://cadir.my.salesforce-sites.com/PagaSearch</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3422,17 +3422,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>NLRB case search</t>
+          <t>CA LWDA PAGA</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Board and Brew / JJ&amp;N</t>
+          <t>20+ other named subjects (JJ&amp;N, BBRG, CCB&amp;B, TWO RIPPERS, etc.)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>No NLRB case surfaced via search</t>
+          <t>Searched full 2016-2026 range; NO PAGA record</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -3442,12 +3442,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>GAP (portal JS)</t>
+          <t>CONFIRMED null (searched-absent)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>https://www.nlrb.gov/search/cases</t>
+          <t>https://cadir.my.salesforce-sites.com/PagaSearch</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3459,35 +3459,146 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Cal/OSHA / OSHA establishment</t>
+          <t>Cal/OSHA + federal OSHA establishment</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Board and Brew</t>
+          <t>Board &amp; Brew (CA + AZ)</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>No CA/AZ Board &amp; Brew citation surfaced. NB: OSHA 'Bbrg Tr, Llc' insp. 1134580.015 is the FLORIDA Bravo Brio entity, NOT a subject</t>
+          <t>No establishment records (CA 2016-2026; AZ Tempe). NB: OSHA 'Bbrg Tr, Llc' 1134580.015 = FLORIDA Bravo Brio, excluded</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1134580.015 (not a subject)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>SEARCH-INFERRED (exclusion)</t>
+          <t>CONFIRMED null</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>https://www.osha.gov/ords/imis/establishment.inspection_detail?id=1134580.015</t>
+          <t>https://www.osha.gov/ords/imis/establishment.html</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>DOL WHD (enforcedata.dol.gov)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>all subjects</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Not machine-readable (JS SPA); no WHD press-release match</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://enforcedata.dol.gov/</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>NLRB case search</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Board and Brew / JJ&amp;N</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>SPA 404 to fetch; no case indexed via site search</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nlrb.gov/search/cases</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CA DLSE / Labor Commissioner</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>all subjects</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>No reachable statewide public judgment search; SD County OLSE dashboard JS</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dir.ca.gov/dlse/</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>2026-07-25</t>
         </is>

</xml_diff>